<commit_message>
Add SQL assignment2 script with 100 queries
</commit_message>
<xml_diff>
--- a/Job Applications.xlsx
+++ b/Job Applications.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guest user\Documents\CARO\CaroGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F36F3E-9C30-44C6-8241-AC47ADE645A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44BA8E19-3367-4314-AEA7-881C2A7100C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BA809F01-3F56-4713-899C-D30734EF9A85}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Company</t>
   </si>
@@ -127,6 +127,21 @@
   </si>
   <si>
     <t>https://jubileeinsurance.com/ke/career/data-governance-intern/</t>
+  </si>
+  <si>
+    <t>DalBerg</t>
+  </si>
+  <si>
+    <t>Data Engineer</t>
+  </si>
+  <si>
+    <t>African Management Institute</t>
+  </si>
+  <si>
+    <t>Content Intern</t>
+  </si>
+  <si>
+    <t>https://careers.africanmanagers.com/jobs/Careers/685437000011728730/Content-Intern-Nairobi-South-Africa-?source=CareerSite</t>
   </si>
 </sst>
 </file>
@@ -192,6 +207,9 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -209,9 +227,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -226,14 +241,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C8A00A5-5BAE-42E0-9DEB-9060E099302C}" name="Table1" displayName="Table1" ref="A1:G9" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:G9" xr:uid="{0C8A00A5-5BAE-42E0-9DEB-9060E099302C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C8A00A5-5BAE-42E0-9DEB-9060E099302C}" name="Table1" displayName="Table1" ref="A1:G11" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:G11" xr:uid="{0C8A00A5-5BAE-42E0-9DEB-9060E099302C}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{155A5FAD-14ED-4D69-AF65-A61E5900B460}" name="Company"/>
     <tableColumn id="2" xr3:uid="{611D0B33-2EDD-4030-A783-93D1C20297EA}" name="Title"/>
     <tableColumn id="3" xr3:uid="{6B28C32E-F4A5-4B4C-9478-06DB431F6B92}" name="Status"/>
     <tableColumn id="4" xr3:uid="{72F9695D-4E9F-4DA4-AF00-9C3F854409C5}" name="Job Posting Link"/>
-    <tableColumn id="5" xr3:uid="{39D71473-DB09-47D6-80E7-C982F226FF46}" name="Application Date" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{39D71473-DB09-47D6-80E7-C982F226FF46}" name="Application Date" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{C0343B25-B301-49B0-814B-38EEABEC3615}" name="Interview Stage"/>
     <tableColumn id="7" xr3:uid="{EDADE3AE-CED9-43C9-BE93-9D2404239EC5}" name="Notes"/>
   </tableColumns>
@@ -538,12 +553,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AEE9600-FF63-4284-8776-D4280E15E424}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="119.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" style="3" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
   </cols>
@@ -707,13 +722,48 @@
         <v>46073</v>
       </c>
     </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46090</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="3">
+        <v>46090</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="https://equitybank.taleo.net/careersection/ext_new/jobdetail.ftl?job=2600002V" xr:uid="{BE455DE2-8442-4555-B982-174DA6D29A8E}"/>
+    <hyperlink ref="D10" r:id="rId2" display="https://join.augmentimpact.ai/apply/310" xr:uid="{972E766B-EE2D-409B-8E04-7E4A2C005654}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>